<commit_message>
fix(TATA receipt): 補齊 Shipper/Volume/完整 MAWB/PPN 擷取
這次使用者提供的新樣本 (GLOSTAR EXPRESS AGUSTUS 2025) 暴露
parse_tata_receipt() 的多個缺口：
- MAWB:/HAWB: 後面帶空格的值 (例如 "738-5567 8873") 被截斷成只抓到
  第一個空白前的片段，改成抓到整行結尾。
- 帳單上其實印了 Shipper ("SHIP :"/"SHIP:") 跟材積 (獨立一行的
  "數量代碼/重量KG(S)" 格式)，舊版完全沒有擷取，新增對應規則。
- PPN 稅金行 (這種帳單印成 "PPN 12% 12.645"，沒有 "Rp" 前綴、跟
  classic 格式不同) 之前完全沒有擷取，新增規則；同時處理版面陷阱
  "PPN 12% 11.0% 332.118" (利率小標籤被擠進同一行) 要取最後一個數字
  才是真正金額。

同步修正 test_samples/YJE_TATA 下 sample3/sample4 這兩份舊版 fixture
(預留的 VAT/Shipper 欄位從未填過，是範本升級缺口，不是程式碼 bug)，
新增 sample8 (GLOSTAR EXPRESS AGUSTUS 2025) 作為新的回歸測試樣本。
全部 8 份樣本重新驗證都達到 100% 正確率，其餘供應商回歸測試無影響
(唯一既有失敗項 INDOPROSTIME/sample1 跟本次改動無關)。

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JhL7qxuxZLsZyoRKZr1of6
</commit_message>
<xml_diff>
--- a/test_samples/YJE_TATA/sample3_ref.xlsx
+++ b/test_samples/YJE_TATA/sample3_ref.xlsx
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <cols>
     <col width="17.36328125" customWidth="1" style="6" min="1" max="1"/>
@@ -608,6 +608,17 @@
 貨櫃號碼</t>
         </is>
       </c>
+      <c r="Q1" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="R1" s="0" t="inlineStr">
+        <is>
+          <t>Shipper
+出貨方</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
@@ -673,7 +684,7 @@
       </c>
       <c r="N2" s="0" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>3CTN/109KG</t>
         </is>
       </c>
       <c r="O2" s="0" t="inlineStr">
@@ -684,6 +695,16 @@
       <c r="P2" s="0" t="inlineStr">
         <is>
           <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q2" s="0" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R2" s="0" t="inlineStr">
+        <is>
+          <t>MYVI TANNERY AND LEATHER PRODUCTS CO.,LTD</t>
         </is>
       </c>
     </row>
@@ -751,7 +772,7 @@
       </c>
       <c r="N3" s="0" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>3CTN/109KG</t>
         </is>
       </c>
       <c r="O3" s="0" t="inlineStr">
@@ -762,6 +783,16 @@
       <c r="P3" s="0" t="inlineStr">
         <is>
           <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q3" s="0" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R3" s="0" t="inlineStr">
+        <is>
+          <t>MYVI TANNERY AND LEATHER PRODUCTS CO.,LTD</t>
         </is>
       </c>
     </row>
@@ -829,7 +860,7 @@
       </c>
       <c r="N4" s="0" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>3CTN/109KG</t>
         </is>
       </c>
       <c r="O4" s="0" t="inlineStr">
@@ -840,6 +871,16 @@
       <c r="P4" s="0" t="inlineStr">
         <is>
           <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q4" s="0" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R4" s="0" t="inlineStr">
+        <is>
+          <t>MYVI TANNERY AND LEATHER PRODUCTS CO.,LTD</t>
         </is>
       </c>
     </row>
@@ -907,7 +948,7 @@
       </c>
       <c r="N5" s="0" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>3CTN/109KG</t>
         </is>
       </c>
       <c r="O5" s="0" t="inlineStr">
@@ -918,6 +959,16 @@
       <c r="P5" s="0" t="inlineStr">
         <is>
           <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q5" s="0" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R5" s="0" t="inlineStr">
+        <is>
+          <t>MYVI TANNERY AND LEATHER PRODUCTS CO.,LTD</t>
         </is>
       </c>
     </row>
@@ -985,7 +1036,7 @@
       </c>
       <c r="N6" s="0" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>3CTN/109KG</t>
         </is>
       </c>
       <c r="O6" s="0" t="inlineStr">
@@ -998,11 +1049,104 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="Q6" s="0" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R6" s="0" t="inlineStr">
+        <is>
+          <t>MYVI TANNERY AND LEATHER PRODUCTS CO.,LTD</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
+      <c r="A7" s="4" t="n">
+        <v>45660</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>TH20250064</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>PT TATA HARMONI SARANATAMA</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>PT GLOSTAR INDONESIA (CJR)</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t>PPN 12%</t>
+        </is>
+      </c>
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G7" s="0" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J7" s="0" t="inlineStr">
+        <is>
+          <t>A2412211-S</t>
+        </is>
+      </c>
+      <c r="K7" s="0" t="inlineStr">
+        <is>
+          <t>978-22076025</t>
+        </is>
+      </c>
+      <c r="L7" s="0" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M7" s="0" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N7" s="0" t="inlineStr">
+        <is>
+          <t>3CTN/109KG</t>
+        </is>
+      </c>
+      <c r="O7" s="0" t="inlineStr">
+        <is>
+          <t>VJ855</t>
+        </is>
+      </c>
+      <c r="P7" s="0" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q7" s="0" t="n">
+        <v>331458</v>
+      </c>
+      <c r="R7" s="0" t="inlineStr">
+        <is>
+          <t>MYVI TANNERY AND LEATHER PRODUCTS CO.,LTD</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n"/>

</xml_diff>